<commit_message>
security: add mini-api authentication-edge cases (secret hygiene)
be-api-mini.feature already covers the token gate (401/403, scopes, IDOR, CORS,
rate-limit). This adds the edges in be-mini-security.feature @security (2 cases,
302-303): a non-Bearer Authorization header is refused (401), and no bearer
token echoes back in a public response (a precise "k_<...>" JSON-value match,
so it does not false-positive on field names like last_block_hash). Both stacks
2/2; no service change.
</commit_message>
<xml_diff>
--- a/testcases/MiniAPI-TestCases.xlsx
+++ b/testcases/MiniAPI-TestCases.xlsx
@@ -3860,7 +3860,122 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C302</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08. API — authentication edges</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Authorization header</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BE/API</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A malformed Authorization header (no Bearer scheme) is 401</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The token check must key on the Bearer scheme, not merely on some header being present</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anvil with a fresh PerpDEX; mini-api running and its indexer caught up</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1) GET /portfolio/summary?account=&lt;any&gt; with header "Authorization: Token k_whatever" (no Bearer scheme) → 401 unauthenticated</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">401 unauthenticated</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C303</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08. API — authentication edges</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">secret hygiene</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BE/API</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public responses never carry a bearer token</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A minted token is returned once at /auth/token and must never echo back in ordinary reads</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anvil with a fresh PerpDEX; mini-api running and its indexer caught up</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1) GET /markets → the JSON body contains no "k_" bearer token
+2) GET /health → the JSON body contains no "k_" bearer token</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No credential in the response bodies</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K67"/>
+  <autoFilter ref="A1:K69"/>
 </worksheet>
 </file>
</xml_diff>